<commit_message>
v0.9-M1: aoa_scale fix, doctor command, physics linter, cache hardening
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,11 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.00000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -77,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -88,10 +85,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +451,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -567,50 +560,6 @@
       <c r="B2" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D2" s="6" t="n">
-        <v>0.1969169152048044</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>0.01826545752819166</v>
-      </c>
-      <c r="F2" s="7" t="n">
-        <v>10.7808</v>
-      </c>
-      <c r="G2" s="8" t="n">
-        <v>48.24464422517708</v>
-      </c>
-      <c r="H2" s="8" t="n">
-        <v>4.475037094406956</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>10.7808</v>
-      </c>
-      <c r="J2" t="n">
-        <v>400</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:08:46</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:20:14</t>
-        </is>
-      </c>
-      <c r="O2" s="9" t="n">
-        <v>11.47</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>runs\cases\r002_aoa0_v20</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -619,50 +568,6 @@
       <c r="B3" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="D3" s="6" t="n">
-        <v>0.1980995888781388</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>0.01749254831178309</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>11.3248</v>
-      </c>
-      <c r="G3" s="8" t="n">
-        <v>109.202398369074</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>9.642767256870428</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>11.3248</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-07-05 21:34:36</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-07-05 22:21:45</t>
-        </is>
-      </c>
-      <c r="O3" s="9" t="n">
-        <v>47.15</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>runs\cases\r003_aoa0_v30</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -671,50 +576,6 @@
       <c r="B4" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D4" s="6" t="n">
-        <v>-0.01462162347098452</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>0.01293909916951414</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>-1.13</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>-3.582297750391207</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>3.170079296530964</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>-1.13</v>
-      </c>
-      <c r="J4" t="n">
-        <v>400</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:25:30</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:36:48</t>
-        </is>
-      </c>
-      <c r="O4" s="9" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>runs\cases\r004_aoa4_v20</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -723,50 +584,6 @@
       <c r="B5" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="D5" s="6" t="n">
-        <v>-0.01453853708395713</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>0.01218945279199403</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>-1.1927</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>-8.014368567531369</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>6.719435851586709</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>-1.1927</v>
-      </c>
-      <c r="J5" t="n">
-        <v>400</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:36:48</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:51:05</t>
-        </is>
-      </c>
-      <c r="O5" s="9" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>runs\cases\r005_aoa4_v30</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -775,50 +592,6 @@
       <c r="B6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>-0.2384074681056423</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>0.02126251441066184</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>-11.2126</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>-58.40982968588236</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>5.209316030612151</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>-11.2126</v>
-      </c>
-      <c r="J6" t="n">
-        <v>300</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-07-04 16:52:50</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:01:21</t>
-        </is>
-      </c>
-      <c r="O6" s="9" t="n">
-        <v>8.529999999999999</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>runs\cases\r006_aoa8_v20</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -827,50 +600,6 @@
       <c r="B7" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>-0.2391490132693947</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0.02056913931312146</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>-11.6266</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>-131.8308935647538</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>11.3387380463582</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>-11.6266</v>
-      </c>
-      <c r="J7" t="n">
-        <v>300</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:01:22</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:09:36</t>
-        </is>
-      </c>
-      <c r="O7" s="9" t="n">
-        <v>8.24</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>runs\cases\r007_aoa8_v30</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -879,50 +608,6 @@
       <c r="B8" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D8" s="6" t="n">
-        <v>-0.4558310368427774</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>0.04251361475810935</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>-10.722</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>-111.6786040264805</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>10.41583561573679</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>-10.722</v>
-      </c>
-      <c r="J8" t="n">
-        <v>300</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:11:49</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:21:50</t>
-        </is>
-      </c>
-      <c r="O8" s="9" t="n">
-        <v>10.02</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>runs\cases\r008_aoa12_v20</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -930,50 +615,6 @@
       </c>
       <c r="B9" s="2" t="n">
         <v>30</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>-0.4563581886288989</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0.04171794168892402</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>-10.9391</v>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>-251.5674514816805</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>22.99701535601937</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>-10.9391</v>
-      </c>
-      <c r="J9" t="n">
-        <v>300</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:21:50</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-07-04 17:32:13</t>
-        </is>
-      </c>
-      <c r="O9" s="9" t="n">
-        <v>10.39</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>runs\cases\r009_aoa12_v30</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -988,7 +629,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="96" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
v0.9-M2: per-iteration telemetry tap, live residuals plot
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -74,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -85,6 +88,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,7 +458,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -560,6 +567,29 @@
       <c r="B2" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>runs\cases\r002_aoa0_v20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -568,6 +598,29 @@
       <c r="B3" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>runs\cases\r003_aoa0_v30</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -576,6 +629,29 @@
       <c r="B4" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>runs\cases\r004_aoa4_v20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -584,6 +660,29 @@
       <c r="B5" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>runs\cases\r005_aoa4_v30</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -592,6 +691,29 @@
       <c r="B6" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>runs\cases\r006_aoa8_v20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -599,6 +721,56 @@
       </c>
       <c r="B7" s="2" t="n">
         <v>30</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>-0.6832828950554133</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.0587689694660613</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>-11.6266</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>-131.8308935647538</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>11.3387380463582</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>-11.6266</v>
+      </c>
+      <c r="J7" t="n">
+        <v>300</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-07-09 01:01:20</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-07-09 01:14:50</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>runs\cases\r007_aoa8_v30</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -629,7 +801,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="96" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
v0.9-M3: SQLite ledger — provenance, per-iteration storage, cross-study queries
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,11 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.00000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -77,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -88,10 +85,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +451,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -567,29 +560,6 @@
       <c r="B2" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>runs\cases\r002_aoa0_v20</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -598,29 +568,6 @@
       <c r="B3" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>runs\cases\r003_aoa0_v30</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -629,29 +576,6 @@
       <c r="B4" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>runs\cases\r004_aoa4_v20</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -660,29 +584,6 @@
       <c r="B5" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>runs\cases\r005_aoa4_v30</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -691,29 +592,6 @@
       <c r="B6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>FluentError: Fluent failed to launch: 'AWP_ROOT271'</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>runs\cases\r006_aoa8_v20</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -721,56 +599,6 @@
       </c>
       <c r="B7" s="2" t="n">
         <v>30</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>-0.6832828950554133</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0.0587689694660613</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>-11.6266</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>-131.8308935647538</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>11.3387380463582</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>-11.6266</v>
-      </c>
-      <c r="J7" t="n">
-        <v>300</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-07-09 01:01:20</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-07-09 01:14:50</t>
-        </is>
-      </c>
-      <c r="O7" s="9" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>runs\cases\r007_aoa8_v30</t>
-        </is>
       </c>
     </row>
     <row r="8">
@@ -801,7 +629,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="96" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat: modernize desktop GUI layout and navigation
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -532,16 +532,16 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:11:06</t>
+          <t>2026-07-23 11:20:00</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:18:50</t>
+          <t>2026-07-23 11:28:41</t>
         </is>
       </c>
       <c r="O2" s="9" t="n">
-        <v>7.73</v>
+        <v>8.69</v>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
@@ -600,16 +600,16 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:18:54</t>
+          <t>2026-07-23 11:28:46</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:26:17</t>
+          <t>2026-07-23 11:37:05</t>
         </is>
       </c>
       <c r="O3" s="9" t="n">
-        <v>7.37</v>
+        <v>8.32</v>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
@@ -636,7 +636,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>RUNNING</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
@@ -702,11 +702,7 @@
       <c r="B5" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C5" s="5" t="n"/>
       <c r="D5" s="6" t="n">
         <v>0.7038256400938724</v>
       </c>
@@ -770,11 +766,7 @@
       <c r="B6" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="6" t="n">
         <v>0.7049291495064187</v>
       </c>
@@ -838,11 +830,7 @@
       <c r="B7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="6" t="n">
         <v>0.7524332178873554</v>
       </c>
@@ -906,11 +894,7 @@
       <c r="B8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C8" s="0" t="n"/>
       <c r="D8" s="6" t="n">
         <v>0.7575765504792562</v>
       </c>
@@ -929,21 +913,21 @@
       <c r="I8" s="7" t="n">
         <v>9.503500000000001</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="0" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
+      <c r="L8" s="0" t="inlineStr"/>
+      <c r="M8" s="0" t="inlineStr">
         <is>
           <t>2026-07-11 20:06:35</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N8" s="0" t="inlineStr">
         <is>
           <t>2026-07-11 20:20:26</t>
         </is>
@@ -951,7 +935,7 @@
       <c r="O8" s="9" t="n">
         <v>13.85</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>runs\cases\r008_aoa10_v10</t>
         </is>
@@ -974,11 +958,7 @@
       <c r="B9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C9" s="5" t="n"/>
       <c r="D9" s="6" t="n">
         <v>0.7602557463596907</v>
       </c>
@@ -1042,11 +1022,7 @@
       <c r="B10" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C10" s="5" t="n"/>
       <c r="D10" s="6" t="n">
         <v>0.7614003715834471</v>
       </c>
@@ -1110,11 +1086,7 @@
       <c r="B11" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
+      <c r="C11" s="5" t="n"/>
       <c r="D11" s="6" t="n">
         <v>0.7626078750625093</v>
       </c>

</xml_diff>

<commit_message>
refactor: integrate runtime with universal platform metadata
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>RUNNING</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
@@ -668,16 +668,16 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:26:19</t>
+          <t>2026-07-23 11:37:13</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:34:03</t>
+          <t>2026-07-23 11:47:24</t>
         </is>
       </c>
       <c r="O4" s="9" t="n">
-        <v>7.74</v>
+        <v>10.19</v>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
@@ -702,7 +702,11 @@
       <c r="B5" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D5" s="6" t="n">
         <v>0.7038256400938724</v>
       </c>
@@ -732,16 +736,16 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:34:07</t>
+          <t>2026-07-23 11:47:30</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:41:48</t>
+          <t>2026-07-23 11:58:34</t>
         </is>
       </c>
       <c r="O5" s="9" t="n">
-        <v>7.68</v>
+        <v>11.06</v>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
@@ -766,7 +770,11 @@
       <c r="B6" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D6" s="6" t="n">
         <v>0.7049291495064187</v>
       </c>
@@ -796,16 +804,16 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:41:51</t>
+          <t>2026-07-23 11:58:43</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:49:45</t>
+          <t>2026-07-23 12:10:12</t>
         </is>
       </c>
       <c r="O6" s="9" t="n">
-        <v>7.9</v>
+        <v>11.48</v>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
@@ -830,7 +838,11 @@
       <c r="B7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n">
         <v>0.7524332178873554</v>
       </c>
@@ -860,16 +872,16 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 19:52:27</t>
+          <t>2026-07-23 12:10:16</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:06:31</t>
+          <t>2026-07-23 12:30:32</t>
         </is>
       </c>
       <c r="O7" s="9" t="n">
-        <v>14.07</v>
+        <v>20.26</v>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
@@ -894,7 +906,11 @@
       <c r="B8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="0" t="n"/>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n">
         <v>0.7575765504792562</v>
       </c>
@@ -924,16 +940,16 @@
       <c r="L8" s="0" t="inlineStr"/>
       <c r="M8" s="0" t="inlineStr">
         <is>
-          <t>2026-07-11 20:06:35</t>
+          <t>2026-07-23 12:30:38</t>
         </is>
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t>2026-07-11 20:20:26</t>
+          <t>2026-07-23 12:49:15</t>
         </is>
       </c>
       <c r="O8" s="9" t="n">
-        <v>13.85</v>
+        <v>18.63</v>
       </c>
       <c r="P8" s="0" t="inlineStr">
         <is>
@@ -958,7 +974,11 @@
       <c r="B9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="C9" s="5" t="n"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D9" s="6" t="n">
         <v>0.7602557463596907</v>
       </c>
@@ -988,16 +1008,16 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:20:29</t>
+          <t>2026-07-23 12:49:22</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:34:35</t>
+          <t>2026-07-23 13:03:26</t>
         </is>
       </c>
       <c r="O9" s="9" t="n">
-        <v>14.09</v>
+        <v>14.08</v>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
@@ -1022,7 +1042,11 @@
       <c r="B10" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="n"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D10" s="6" t="n">
         <v>0.7614003715834471</v>
       </c>
@@ -1052,16 +1076,16 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:34:39</t>
+          <t>2026-07-23 13:03:31</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:48:49</t>
+          <t>2026-07-23 13:16:16</t>
         </is>
       </c>
       <c r="O10" s="9" t="n">
-        <v>14.18</v>
+        <v>12.77</v>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
@@ -1086,7 +1110,11 @@
       <c r="B11" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C11" s="5" t="n"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="n">
         <v>0.7626078750625093</v>
       </c>
@@ -1116,16 +1144,16 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 20:48:53</t>
+          <t>2026-07-23 13:16:21</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11 21:03:11</t>
+          <t>2026-07-23 13:30:32</t>
         </is>
       </c>
       <c r="O11" s="9" t="n">
-        <v>14.29</v>
+        <v>14.19</v>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: implement project template selection
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -906,7 +906,7 @@
       <c r="B8" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -929,21 +929,21 @@
       <c r="I8" s="9" t="n">
         <v>7.3497</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="0" t="n">
         <v>1500</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="0" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
+      <c r="L8" s="0" t="inlineStr"/>
+      <c r="M8" s="0" t="inlineStr">
         <is>
           <t>2026-07-24 04:33:58</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N8" s="0" t="inlineStr">
         <is>
           <t>2026-07-24 05:41:59</t>
         </is>
@@ -951,7 +951,7 @@
       <c r="O8" s="11" t="n">
         <v>68.02</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>runs\cases\r008_aoa15_v10</t>
         </is>
@@ -1518,20 +1518,56 @@
       <c r="B17" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="9" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="4" t="n"/>
-      <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="7" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>1.102461114752772</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>0.1652994195548312</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>6.6695</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>16.88143581965182</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>2.531147361933353</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>6.6695</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:22:51</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:43:08</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="n">
+        <v>20.29</v>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>runs\cases\r017_aoa17_v5</t>
+        </is>
+      </c>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="4" t="n"/>
       <c r="S17" s="4" t="n"/>
@@ -1550,20 +1586,56 @@
       <c r="B18" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="9" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4" t="n"/>
-      <c r="O18" s="11" t="n"/>
-      <c r="P18" s="4" t="n"/>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>1.111476937529324</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>0.1644586909247591</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>6.7584</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>68.0779624236711</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>10.0730948191415</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>6.7584</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>800</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:43:14</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:54:30</t>
+        </is>
+      </c>
+      <c r="O18" s="11" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r018_aoa17_v10</t>
+        </is>
+      </c>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="4" t="n"/>
       <c r="S18" s="4" t="n"/>
@@ -1582,20 +1654,56 @@
       <c r="B19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="9" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="11" t="n"/>
-      <c r="P19" s="4" t="n"/>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>1.115263928075961</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>0.1640251138027081</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>6.7993</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>153.6973100879684</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>22.60471099593571</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>6.7993</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:54:36</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:08:34</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="n">
+        <v>13.97</v>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r019_aoa17_v15</t>
+        </is>
+      </c>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
       <c r="S19" s="4" t="n"/>
@@ -1614,20 +1722,56 @@
       <c r="B20" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="9" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
-      <c r="N20" s="4" t="n"/>
-      <c r="O20" s="11" t="n"/>
-      <c r="P20" s="4" t="n"/>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1.118319789371935</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>0.1640042440171021</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>6.8188</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>273.9883483961241</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>40.18103978419001</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>6.8188</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:08:42</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:24:57</t>
+        </is>
+      </c>
+      <c r="O20" s="11" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r020_aoa17_v20</t>
+        </is>
+      </c>
       <c r="Q20" s="4" t="n"/>
       <c r="R20" s="4" t="n"/>
       <c r="S20" s="4" t="n"/>
@@ -1646,20 +1790,56 @@
       <c r="B21" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="9" t="n"/>
-      <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="n"/>
-      <c r="L21" s="4" t="n"/>
-      <c r="M21" s="4" t="n"/>
-      <c r="N21" s="4" t="n"/>
-      <c r="O21" s="11" t="n"/>
-      <c r="P21" s="4" t="n"/>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>1.118786578633382</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>0.1634194599316674</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>6.8461</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>428.2854871330916</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>62.55901200509143</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>6.8461</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:25:07</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:38:17</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r021_aoa17_v25</t>
+        </is>
+      </c>
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="4" t="n"/>
       <c r="S21" s="4" t="n"/>
@@ -1678,20 +1858,56 @@
       <c r="B22" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="10" t="n"/>
-      <c r="I22" s="9" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="n"/>
-      <c r="M22" s="4" t="n"/>
-      <c r="N22" s="4" t="n"/>
-      <c r="O22" s="11" t="n"/>
-      <c r="P22" s="4" t="n"/>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>1.154270425532516</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>0.1813795865531983</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>6.3638</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>17.67476589096665</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>2.777374919095849</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>6.3638</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:42:33</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:03:29</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r022_aoa18_v5</t>
+        </is>
+      </c>
       <c r="Q22" s="4" t="n"/>
       <c r="R22" s="4" t="n"/>
       <c r="S22" s="4" t="n"/>
@@ -1710,20 +1926,56 @@
       <c r="B23" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="10" t="n"/>
-      <c r="I23" s="9" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n"/>
-      <c r="M23" s="4" t="n"/>
-      <c r="N23" s="4" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="4" t="n"/>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>1.162560200333631</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>0.1803913295316586</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>6.4447</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>71.2068122704349</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>11.04896893381409</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>6.4447</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:03:35</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:16:21</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="n">
+        <v>12.77</v>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r023_aoa18_v10</t>
+        </is>
+      </c>
       <c r="Q23" s="4" t="n"/>
       <c r="R23" s="4" t="n"/>
       <c r="S23" s="4" t="n"/>
@@ -1742,20 +1994,56 @@
       <c r="B24" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="9" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="10" t="n"/>
-      <c r="I24" s="9" t="n"/>
-      <c r="J24" s="4" t="n"/>
-      <c r="K24" s="4" t="n"/>
-      <c r="L24" s="4" t="n"/>
-      <c r="M24" s="4" t="n"/>
-      <c r="N24" s="4" t="n"/>
-      <c r="O24" s="11" t="n"/>
-      <c r="P24" s="4" t="n"/>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>1.167067941251508</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>0.1801540242370069</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>6.4782</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>160.8365506537234</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>24.82747646516252</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>6.4782</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:16:28</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:30:54</t>
+        </is>
+      </c>
+      <c r="O24" s="11" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r024_aoa18_v15</t>
+        </is>
+      </c>
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="4" t="n"/>
       <c r="S24" s="4" t="n"/>
@@ -1774,20 +2062,56 @@
       <c r="B25" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="10" t="n"/>
-      <c r="I25" s="9" t="n"/>
-      <c r="J25" s="4" t="n"/>
-      <c r="K25" s="4" t="n"/>
-      <c r="L25" s="4" t="n"/>
-      <c r="M25" s="4" t="n"/>
-      <c r="N25" s="4" t="n"/>
-      <c r="O25" s="11" t="n"/>
-      <c r="P25" s="4" t="n"/>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>1.16946987816508</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>0.1799003316993219</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>6.5007</v>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>286.5201201504446</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>44.07558126633386</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>6.5007</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 15:31:01</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 16:28:04</t>
+        </is>
+      </c>
+      <c r="O25" s="11" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r025_aoa18_v20</t>
+        </is>
+      </c>
       <c r="Q25" s="4" t="n"/>
       <c r="R25" s="4" t="n"/>
       <c r="S25" s="4" t="n"/>
@@ -1806,20 +2130,56 @@
       <c r="B26" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="10" t="n"/>
-      <c r="I26" s="9" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="11" t="n"/>
-      <c r="P26" s="4" t="n"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>1.17110748262434</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0.1797694902504477</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>6.5145</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>448.3145831921302</v>
+      </c>
+      <c r="H26" s="10" t="n">
+        <v>68.81800798649952</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>6.5145</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 16:28:12</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24 16:42:29</t>
+        </is>
+      </c>
+      <c r="O26" s="11" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>runs\cases\r026_aoa18_v25</t>
+        </is>
+      </c>
       <c r="Q26" s="4" t="n"/>
       <c r="R26" s="4" t="n"/>
       <c r="S26" s="4" t="n"/>

</xml_diff>